<commit_message>
Complete EDA and preprocessing
</commit_message>
<xml_diff>
--- a/data/competitive_matches.xlsx
+++ b/data/competitive_matches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\valorant_personal_coach\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2127E6E-C5B4-47C7-9160-AAB73FDBB7BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1832BCF-60CC-4973-80DC-84E8BAE49F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="58">
   <si>
     <t>VALORANT Personal Coach — Competitive Match History</t>
   </si>
@@ -217,7 +217,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -237,6 +237,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -262,8 +268,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -284,15 +291,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -534,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X299"/>
+  <dimension ref="A1:X306"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -554,30 +562,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" s="5" customFormat="1" ht="25.9" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="9"/>
+      <c r="V1" s="9"/>
       <c r="X1" s="6" t="s">
         <v>1</v>
       </c>
@@ -649,7 +657,7 @@
       <c r="V2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X2" s="8" t="s">
+      <c r="X2" s="10" t="s">
         <v>23</v>
       </c>
     </row>
@@ -20131,19 +20139,19 @@
         <v>8</v>
       </c>
       <c r="H259" s="1" t="str">
-        <f t="shared" ref="H259:H299" si="32">IF(F259&gt;G259,"Win",IF(F259&lt;G259,"Loss","Draw"))</f>
+        <f t="shared" ref="H259:H306" si="32">IF(F259&gt;G259,"Win",IF(F259&lt;G259,"Loss","Draw"))</f>
         <v>Win</v>
       </c>
       <c r="I259" s="1">
-        <f t="shared" ref="I259:I299" si="33">IF(H259="Win",1,IF(H259="Loss",0,""))</f>
+        <f t="shared" ref="I259:I306" si="33">IF(H259="Win",1,IF(H259="Loss",0,""))</f>
         <v>1</v>
       </c>
       <c r="J259" s="1">
-        <f t="shared" ref="J259:J299" si="34">F259-G259</f>
+        <f t="shared" ref="J259:J306" si="34">F259-G259</f>
         <v>5</v>
       </c>
       <c r="K259" s="1">
-        <f t="shared" ref="K259:K299" si="35">F259+G259</f>
+        <f t="shared" ref="K259:K306" si="35">F259+G259</f>
         <v>21</v>
       </c>
       <c r="L259" s="1">
@@ -20156,19 +20164,19 @@
         <v>9</v>
       </c>
       <c r="O259" s="3">
-        <f t="shared" ref="O259:O299" si="36">IF(M259=0,"",L259/M259)</f>
+        <f t="shared" ref="O259:O306" si="36">IF(M259=0,"",L259/M259)</f>
         <v>1</v>
       </c>
       <c r="P259" s="3">
-        <f t="shared" ref="P259:P299" si="37">IF(K259=0,"",L259/K259)</f>
+        <f t="shared" ref="P259:P306" si="37">IF(K259=0,"",L259/K259)</f>
         <v>0.80952380952380953</v>
       </c>
       <c r="Q259" s="3">
-        <f t="shared" ref="Q259:Q299" si="38">IF(K259=0,"",M259/K259)</f>
+        <f t="shared" ref="Q259:Q306" si="38">IF(K259=0,"",M259/K259)</f>
         <v>0.80952380952380953</v>
       </c>
       <c r="R259" s="3">
-        <f t="shared" ref="R259:R299" si="39">IF(K259=0,"",N259/K259)</f>
+        <f t="shared" ref="R259:R306" si="39">IF(K259=0,"",N259/K259)</f>
         <v>0.42857142857142855</v>
       </c>
       <c r="S259" s="1">
@@ -23152,7 +23160,7 @@
       <c r="A299" s="1">
         <v>297</v>
       </c>
-      <c r="B299" s="9">
+      <c r="B299" s="8">
         <v>46285</v>
       </c>
       <c r="C299" s="1" t="s">
@@ -23222,13 +23230,545 @@
       </c>
       <c r="V299" s="1">
         <v>606</v>
+      </c>
+    </row>
+    <row r="300" spans="1:22">
+      <c r="A300" s="1">
+        <v>298</v>
+      </c>
+      <c r="B300" s="8">
+        <v>46290</v>
+      </c>
+      <c r="C300" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D300" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E300" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F300" s="1">
+        <v>3</v>
+      </c>
+      <c r="G300" s="1">
+        <v>13</v>
+      </c>
+      <c r="H300" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Loss</v>
+      </c>
+      <c r="I300" s="1">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="J300" s="1">
+        <f t="shared" si="34"/>
+        <v>-10</v>
+      </c>
+      <c r="K300" s="1">
+        <f t="shared" si="35"/>
+        <v>16</v>
+      </c>
+      <c r="L300" s="1">
+        <v>4</v>
+      </c>
+      <c r="M300" s="1">
+        <v>14</v>
+      </c>
+      <c r="N300" s="1">
+        <v>6</v>
+      </c>
+      <c r="O300" s="3">
+        <f t="shared" si="36"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="P300" s="3">
+        <f t="shared" si="37"/>
+        <v>0.25</v>
+      </c>
+      <c r="Q300" s="3">
+        <f t="shared" si="38"/>
+        <v>0.875</v>
+      </c>
+      <c r="R300" s="3">
+        <f t="shared" si="39"/>
+        <v>0.375</v>
+      </c>
+      <c r="S300" s="1">
+        <v>-91</v>
+      </c>
+      <c r="T300" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="U300" s="1">
+        <v>104</v>
+      </c>
+      <c r="V300" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="301" spans="1:22">
+      <c r="A301" s="1">
+        <v>299</v>
+      </c>
+      <c r="B301" s="8">
+        <v>46291</v>
+      </c>
+      <c r="C301" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D301" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E301" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F301" s="1">
+        <v>13</v>
+      </c>
+      <c r="G301" s="1">
+        <v>7</v>
+      </c>
+      <c r="H301" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Win</v>
+      </c>
+      <c r="I301" s="1">
+        <f t="shared" si="33"/>
+        <v>1</v>
+      </c>
+      <c r="J301" s="1">
+        <f t="shared" si="34"/>
+        <v>6</v>
+      </c>
+      <c r="K301" s="1">
+        <f t="shared" si="35"/>
+        <v>20</v>
+      </c>
+      <c r="L301" s="1">
+        <v>18</v>
+      </c>
+      <c r="M301" s="1">
+        <v>10</v>
+      </c>
+      <c r="N301" s="1">
+        <v>0</v>
+      </c>
+      <c r="O301" s="3">
+        <f t="shared" si="36"/>
+        <v>1.8</v>
+      </c>
+      <c r="P301" s="3">
+        <f t="shared" si="37"/>
+        <v>0.9</v>
+      </c>
+      <c r="Q301" s="3">
+        <f t="shared" si="38"/>
+        <v>0.5</v>
+      </c>
+      <c r="R301" s="3">
+        <f t="shared" si="39"/>
+        <v>0</v>
+      </c>
+      <c r="S301" s="1">
+        <v>38</v>
+      </c>
+      <c r="T301" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="U301" s="1">
+        <v>234</v>
+      </c>
+      <c r="V301" s="1">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="302" spans="1:22">
+      <c r="A302" s="1">
+        <v>300</v>
+      </c>
+      <c r="B302" s="8">
+        <v>46291</v>
+      </c>
+      <c r="C302" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D302" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E302" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F302" s="1">
+        <v>13</v>
+      </c>
+      <c r="G302" s="1">
+        <v>8</v>
+      </c>
+      <c r="H302" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Win</v>
+      </c>
+      <c r="I302" s="1">
+        <f t="shared" si="33"/>
+        <v>1</v>
+      </c>
+      <c r="J302" s="1">
+        <f t="shared" si="34"/>
+        <v>5</v>
+      </c>
+      <c r="K302" s="1">
+        <f t="shared" si="35"/>
+        <v>21</v>
+      </c>
+      <c r="L302" s="1">
+        <v>12</v>
+      </c>
+      <c r="M302" s="1">
+        <v>11</v>
+      </c>
+      <c r="N302" s="1">
+        <v>4</v>
+      </c>
+      <c r="O302" s="3">
+        <f t="shared" si="36"/>
+        <v>1.0909090909090908</v>
+      </c>
+      <c r="P302" s="3">
+        <f t="shared" si="37"/>
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="Q302" s="3">
+        <f t="shared" si="38"/>
+        <v>0.52380952380952384</v>
+      </c>
+      <c r="R302" s="3">
+        <f t="shared" si="39"/>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="S302" s="1">
+        <v>-2</v>
+      </c>
+      <c r="T302" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="U302" s="1">
+        <v>148</v>
+      </c>
+      <c r="V302" s="1">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="303" spans="1:22">
+      <c r="A303" s="1">
+        <v>301</v>
+      </c>
+      <c r="B303" s="8">
+        <v>46291</v>
+      </c>
+      <c r="C303" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D303" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E303" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F303" s="1">
+        <v>6</v>
+      </c>
+      <c r="G303" s="1">
+        <v>11</v>
+      </c>
+      <c r="H303" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Loss</v>
+      </c>
+      <c r="I303" s="1">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="J303" s="1">
+        <f t="shared" si="34"/>
+        <v>-5</v>
+      </c>
+      <c r="K303" s="1">
+        <f t="shared" si="35"/>
+        <v>17</v>
+      </c>
+      <c r="L303" s="1">
+        <v>6</v>
+      </c>
+      <c r="M303" s="1">
+        <v>11</v>
+      </c>
+      <c r="N303" s="1">
+        <v>4</v>
+      </c>
+      <c r="O303" s="3">
+        <f t="shared" si="36"/>
+        <v>0.54545454545454541</v>
+      </c>
+      <c r="P303" s="3">
+        <f t="shared" si="37"/>
+        <v>0.35294117647058826</v>
+      </c>
+      <c r="Q303" s="3">
+        <f t="shared" si="38"/>
+        <v>0.6470588235294118</v>
+      </c>
+      <c r="R303" s="3">
+        <f t="shared" si="39"/>
+        <v>0.23529411764705882</v>
+      </c>
+      <c r="S303" s="1">
+        <v>-43</v>
+      </c>
+      <c r="T303" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="U303" s="1">
+        <v>98</v>
+      </c>
+      <c r="V303" s="1">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="304" spans="1:22">
+      <c r="A304" s="1">
+        <v>302</v>
+      </c>
+      <c r="B304" s="8">
+        <v>46291</v>
+      </c>
+      <c r="C304" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D304" t="s">
+        <v>32</v>
+      </c>
+      <c r="E304" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F304" s="1">
+        <v>13</v>
+      </c>
+      <c r="G304" s="1">
+        <v>9</v>
+      </c>
+      <c r="H304" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Win</v>
+      </c>
+      <c r="I304" s="1">
+        <f t="shared" si="33"/>
+        <v>1</v>
+      </c>
+      <c r="J304" s="1">
+        <f t="shared" si="34"/>
+        <v>4</v>
+      </c>
+      <c r="K304" s="1">
+        <f t="shared" si="35"/>
+        <v>22</v>
+      </c>
+      <c r="L304" s="1">
+        <v>18</v>
+      </c>
+      <c r="M304" s="1">
+        <v>16</v>
+      </c>
+      <c r="N304" s="1">
+        <v>10</v>
+      </c>
+      <c r="O304" s="3">
+        <f t="shared" si="36"/>
+        <v>1.125</v>
+      </c>
+      <c r="P304" s="3">
+        <f t="shared" si="37"/>
+        <v>0.81818181818181823</v>
+      </c>
+      <c r="Q304" s="3">
+        <f t="shared" si="38"/>
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="R304" s="3">
+        <f t="shared" si="39"/>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="S304" s="1">
+        <v>4</v>
+      </c>
+      <c r="T304" s="4">
+        <v>0.06</v>
+      </c>
+      <c r="U304" s="1">
+        <v>238</v>
+      </c>
+      <c r="V304" s="1">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="305" spans="1:22">
+      <c r="A305" s="1">
+        <v>303</v>
+      </c>
+      <c r="B305" s="8">
+        <v>46292</v>
+      </c>
+      <c r="C305" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D305" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E305" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F305" s="1">
+        <v>13</v>
+      </c>
+      <c r="G305" s="1">
+        <v>9</v>
+      </c>
+      <c r="H305" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Win</v>
+      </c>
+      <c r="I305" s="1">
+        <f t="shared" si="33"/>
+        <v>1</v>
+      </c>
+      <c r="J305" s="1">
+        <f t="shared" si="34"/>
+        <v>4</v>
+      </c>
+      <c r="K305" s="1">
+        <f t="shared" si="35"/>
+        <v>22</v>
+      </c>
+      <c r="L305" s="1">
+        <v>7</v>
+      </c>
+      <c r="M305" s="1">
+        <v>15</v>
+      </c>
+      <c r="N305" s="1">
+        <v>11</v>
+      </c>
+      <c r="O305" s="3">
+        <f t="shared" si="36"/>
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="P305" s="3">
+        <f t="shared" si="37"/>
+        <v>0.31818181818181818</v>
+      </c>
+      <c r="Q305" s="3">
+        <f t="shared" si="38"/>
+        <v>0.68181818181818177</v>
+      </c>
+      <c r="R305" s="3">
+        <f t="shared" si="39"/>
+        <v>0.5</v>
+      </c>
+      <c r="S305" s="1">
+        <v>-48</v>
+      </c>
+      <c r="T305" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="U305" s="1">
+        <v>105</v>
+      </c>
+      <c r="V305" s="1">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="306" spans="1:22">
+      <c r="A306" s="1">
+        <v>304</v>
+      </c>
+      <c r="B306" s="8">
+        <v>46292</v>
+      </c>
+      <c r="C306" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D306" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E306" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F306" s="1">
+        <v>11</v>
+      </c>
+      <c r="G306" s="1">
+        <v>13</v>
+      </c>
+      <c r="H306" s="1" t="str">
+        <f t="shared" si="32"/>
+        <v>Loss</v>
+      </c>
+      <c r="I306" s="1">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="J306" s="1">
+        <f t="shared" si="34"/>
+        <v>-2</v>
+      </c>
+      <c r="K306" s="1">
+        <f t="shared" si="35"/>
+        <v>24</v>
+      </c>
+      <c r="L306" s="1">
+        <v>4</v>
+      </c>
+      <c r="M306" s="1">
+        <v>21</v>
+      </c>
+      <c r="N306" s="1">
+        <v>11</v>
+      </c>
+      <c r="O306" s="3">
+        <f t="shared" si="36"/>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="P306" s="3">
+        <f t="shared" si="37"/>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="Q306" s="3">
+        <f t="shared" si="38"/>
+        <v>0.875</v>
+      </c>
+      <c r="R306" s="3">
+        <f t="shared" si="39"/>
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="S306" s="1">
+        <v>-75</v>
+      </c>
+      <c r="T306" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="U306" s="1">
+        <v>90</v>
+      </c>
+      <c r="V306" s="1">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:V1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H3:H299">
+  <conditionalFormatting sqref="H3:H306">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>H3="Win"</formula>
     </cfRule>
@@ -23239,6 +23779,9 @@
       <formula>H3="Draw"</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1" xr:uid="{7743B3AF-FE80-4483-AAA0-A84BFF8731E3}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>